<commit_message>
penyempurnaan fitur import excel
</commit_message>
<xml_diff>
--- a/public/uploads/template/TEMPLATE_INPUT_DATA_BUKU_SILALA_NEW.xlsx
+++ b/public/uploads/template/TEMPLATE_INPUT_DATA_BUKU_SILALA_NEW.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\USER\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\SILALA_BPMSPH\public\uploads\template\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{EA9D724D-040F-49E6-913B-8213DD301183}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{9D25B5F2-8F4E-4C20-BE80-584278FEDDBB}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7545" xr2:uid="{02BECEC1-03E0-47A7-834F-380D8E776085}"/>
   </bookViews>
@@ -27,24 +27,15 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
   <si>
-    <t>File buku URL (PDF)</t>
-  </si>
-  <si>
     <t>penulis</t>
   </si>
   <si>
     <t>penerbit</t>
   </si>
   <si>
-    <t>tahun_Terbit</t>
-  </si>
-  <si>
     <t>bahasa</t>
   </si>
   <si>
-    <t>kategori</t>
-  </si>
-  <si>
     <t>jumlah Halaman</t>
   </si>
   <si>
@@ -57,10 +48,19 @@
     <t>judul_buku</t>
   </si>
   <si>
-    <t>stok_Buku</t>
-  </si>
-  <si>
-    <t>Foto Buku (URL)</t>
+    <t>tahun_terbit</t>
+  </si>
+  <si>
+    <t>data_kategori</t>
+  </si>
+  <si>
+    <t>file_buku URL (PDF)</t>
+  </si>
+  <si>
+    <t>stok</t>
+  </si>
+  <si>
+    <t xml:space="preserve">foto_buku </t>
   </si>
 </sst>
 </file>
@@ -437,40 +437,40 @@
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="F1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>4</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>7</v>
       </c>
       <c r="I1" s="1" t="s">
         <v>10</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="K1" s="1" t="s">
         <v>11</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>0</v>
+        <v>9</v>
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.25">

</xml_diff>